<commit_message>
update qwen3 FSDP2 operator breakdown (best 634ms: AITER attn + fused RMSNorm + fused RoPE)
</commit_message>
<xml_diff>
--- a/examples/qwen3/results/qwen3_fsdp2_operator_breakdown.xlsx
+++ b/examples/qwen3/results/qwen3_fsdp2_operator_breakdown.xlsx
@@ -11,7 +11,7 @@
     <sheet name="算子明细" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="说明" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Roofline-best" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="单算子明细(AITER attn)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="单算子明细(best)" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -453,7 +453,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>来源: chrome trace (step 15-17, 3 steps) | 8×MI308X | GPU kernel self-time. param-storage wall≈1419ms (GPU self 1548ms/step); best+AITER-attn wall≈681ms (GPU self 703ms/step)</t>
+          <t>来源: chrome trace (step 15-17, 3 steps) | 8×MI308X | GPU kernel self-time. param-storage wall≈1419ms (GPU self 1548ms/step); best wall≈634ms (AITER attn+融合RMSNorm/RoPE) (GPU self 657ms/step)</t>
         </is>
       </c>
     </row>
@@ -502,13 +502,13 @@
         <v>490.8</v>
       </c>
       <c r="D5" t="n">
-        <v>1640</v>
+        <v>1068</v>
       </c>
       <c r="E5" t="n">
-        <v>60.7</v>
+        <v>37.1</v>
       </c>
       <c r="F5" t="n">
-        <v>-430.1</v>
+        <v>-453.7</v>
       </c>
     </row>
     <row r="6">
@@ -524,13 +524,13 @@
         <v>421.9</v>
       </c>
       <c r="D6" t="n">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="E6" t="n">
-        <v>302.1</v>
+        <v>296</v>
       </c>
       <c r="F6" t="n">
-        <v>-119.8</v>
+        <v>-125.9</v>
       </c>
     </row>
     <row r="7">
@@ -549,10 +549,10 @@
         <v>144</v>
       </c>
       <c r="E7" t="n">
-        <v>57.5</v>
+        <v>59</v>
       </c>
       <c r="F7" t="n">
-        <v>-128.4</v>
+        <v>-126.9</v>
       </c>
     </row>
     <row r="8">
@@ -568,13 +568,13 @@
         <v>170.1</v>
       </c>
       <c r="D8" t="n">
-        <v>4774</v>
+        <v>1825</v>
       </c>
       <c r="E8" t="n">
-        <v>121.2</v>
+        <v>50.7</v>
       </c>
       <c r="F8" t="n">
-        <v>-48.9</v>
+        <v>-119.4</v>
       </c>
     </row>
     <row r="9">
@@ -590,13 +590,13 @@
         <v>121.8</v>
       </c>
       <c r="D9" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E9" t="n">
-        <v>66.3</v>
+        <v>71.09999999999999</v>
       </c>
       <c r="F9" t="n">
-        <v>-55.5</v>
+        <v>-50.7</v>
       </c>
     </row>
     <row r="10">
@@ -612,139 +612,183 @@
         <v>72.2</v>
       </c>
       <c r="D10" t="n">
-        <v>1510</v>
+        <v>1513</v>
       </c>
       <c r="E10" t="n">
-        <v>49.4</v>
+        <v>54</v>
       </c>
       <c r="F10" t="n">
-        <v>-22.8</v>
+        <v>-18.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>dropout</t>
+          <t>RMSNorm (融合)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>504</v>
+        <v>0</v>
       </c>
       <c r="C11" t="n">
-        <v>29.9</v>
+        <v>0</v>
       </c>
       <c r="D11" t="n">
-        <v>252</v>
+        <v>435</v>
       </c>
       <c r="E11" t="n">
-        <v>14.1</v>
+        <v>42.2</v>
       </c>
       <c r="F11" t="n">
-        <v>-15.8</v>
+        <v>42.2</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FP8 量化</t>
+          <t>dropout</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>758</v>
+        <v>504</v>
       </c>
       <c r="C12" t="n">
-        <v>27.4</v>
+        <v>29.9</v>
       </c>
       <c r="D12" t="n">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="E12" t="n">
-        <v>12.9</v>
+        <v>17.4</v>
       </c>
       <c r="F12" t="n">
-        <v>-14.5</v>
+        <v>-12.5</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>reduce (norm/softmax/sum)</t>
+          <t>FP8 量化</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>439</v>
+        <v>758</v>
       </c>
       <c r="C13" t="n">
-        <v>16.4</v>
+        <v>27.4</v>
       </c>
       <c r="D13" t="n">
-        <v>366</v>
+        <v>253</v>
       </c>
       <c r="E13" t="n">
-        <v>13.1</v>
+        <v>13</v>
       </c>
       <c r="F13" t="n">
-        <v>-3.3</v>
+        <v>-14.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>reduce (norm/softmax/sum)</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>583</v>
+        <v>439</v>
       </c>
       <c r="C14" t="n">
-        <v>10.4</v>
+        <v>16.4</v>
       </c>
       <c r="D14" t="n">
-        <v>294</v>
+        <v>77</v>
       </c>
       <c r="E14" t="n">
-        <v>5.2</v>
+        <v>4.5</v>
       </c>
       <c r="F14" t="n">
-        <v>-5.2</v>
+        <v>-11.9</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>583</v>
+      </c>
+      <c r="C15" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="D15" t="n">
+        <v>295</v>
+      </c>
+      <c r="E15" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="F15" t="n">
+        <v>-4.5</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>RoPE (融合)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" t="n">
+        <v>144</v>
+      </c>
+      <c r="E16" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="F16" t="n">
+        <v>5.4</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>优化器</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B17" t="n">
         <v>69</v>
       </c>
-      <c r="C15" t="n">
+      <c r="C17" t="n">
         <v>0.8</v>
       </c>
-      <c r="D15" t="n">
-        <v>69</v>
-      </c>
-      <c r="E15" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="F15" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="inlineStr">
+      <c r="D17" t="n">
+        <v>87</v>
+      </c>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t>合计 (GPU self-time)</t>
         </is>
       </c>
-      <c r="C16" s="3" t="n">
+      <c r="C18" s="3" t="n">
         <v>1547.7</v>
       </c>
-      <c r="E16" s="3" t="n">
-        <v>703.3</v>
-      </c>
-      <c r="F16" s="3" t="n">
-        <v>-844.4</v>
+      <c r="E18" s="3" t="n">
+        <v>657.4</v>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>-890.3</v>
       </c>
     </row>
   </sheetData>
@@ -758,7 +802,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -843,10 +887,10 @@
         <v>31.5</v>
       </c>
       <c r="E3" t="n">
-        <v>291</v>
+        <v>2</v>
       </c>
       <c r="F3" t="n">
-        <v>18.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -867,10 +911,10 @@
         <v>24.6</v>
       </c>
       <c r="E4" t="n">
-        <v>252</v>
+        <v>324</v>
       </c>
       <c r="F4" t="n">
-        <v>6.7</v>
+        <v>12.2</v>
       </c>
     </row>
     <row r="5">
@@ -894,7 +938,7 @@
         <v>37</v>
       </c>
       <c r="F5" t="n">
-        <v>13.3</v>
+        <v>13.4</v>
       </c>
     </row>
     <row r="6">
@@ -915,10 +959,10 @@
         <v>10.5</v>
       </c>
       <c r="E6" t="n">
-        <v>328</v>
+        <v>40</v>
       </c>
       <c r="F6" t="n">
-        <v>6.1</v>
+        <v>0.2</v>
       </c>
     </row>
     <row r="7">
@@ -939,10 +983,10 @@
         <v>9.800000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>144</v>
+        <v>72</v>
       </c>
       <c r="F7" t="n">
-        <v>7</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="8">
@@ -963,10 +1007,10 @@
         <v>411.5</v>
       </c>
       <c r="E8" t="n">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="F8" t="n">
-        <v>291.7</v>
+        <v>285.6</v>
       </c>
     </row>
     <row r="9">
@@ -1110,7 +1154,7 @@
         <v>36</v>
       </c>
       <c r="F14" t="n">
-        <v>15.8</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="15">
@@ -1155,10 +1199,10 @@
         <v>33.4</v>
       </c>
       <c r="E16" t="n">
-        <v>577</v>
+        <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>21.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -1179,10 +1223,10 @@
         <v>24.6</v>
       </c>
       <c r="E17" t="n">
-        <v>858</v>
+        <v>755</v>
       </c>
       <c r="F17" t="n">
-        <v>18.7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="18">
@@ -1203,10 +1247,10 @@
         <v>22.1</v>
       </c>
       <c r="E18" t="n">
-        <v>362</v>
+        <v>1</v>
       </c>
       <c r="F18" t="n">
-        <v>13.3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1230,7 +1274,7 @@
         <v>505</v>
       </c>
       <c r="F19" t="n">
-        <v>10.1</v>
+        <v>10.8</v>
       </c>
     </row>
     <row r="20">
@@ -1275,10 +1319,10 @@
         <v>8</v>
       </c>
       <c r="E21" t="n">
-        <v>108</v>
+        <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="22">
@@ -1299,10 +1343,10 @@
         <v>121.8</v>
       </c>
       <c r="E22" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F22" t="n">
-        <v>66.3</v>
+        <v>71.09999999999999</v>
       </c>
     </row>
     <row r="23">
@@ -1326,7 +1370,7 @@
         <v>108</v>
       </c>
       <c r="F23" t="n">
-        <v>6.8</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="24">
@@ -1350,7 +1394,7 @@
         <v>72</v>
       </c>
       <c r="F24" t="n">
-        <v>6.1</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="25">
@@ -1374,7 +1418,7 @@
         <v>216</v>
       </c>
       <c r="F25" t="n">
-        <v>4.7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="26">
@@ -1395,7 +1439,7 @@
         <v>7.9</v>
       </c>
       <c r="E26" t="n">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F26" t="n">
         <v>7.5</v>
@@ -1422,7 +1466,7 @@
         <v>252</v>
       </c>
       <c r="F27" t="n">
-        <v>5.8</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="28">
@@ -1446,175 +1490,175 @@
         <v>216</v>
       </c>
       <c r="F28" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>dropout</t>
+          <t>RMSNorm (融合)</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>void at::native::(anonymous namespace)::fused_dropout_kernel</t>
+          <t>_rmsnorm_bwd_triton</t>
         </is>
       </c>
       <c r="C29" t="n">
-        <v>504</v>
+        <v>0</v>
       </c>
       <c r="D29" t="n">
-        <v>29.9</v>
+        <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>252</v>
+        <v>145</v>
       </c>
       <c r="F29" t="n">
-        <v>14.1</v>
+        <v>36.4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>FP8 量化</t>
+          <t>RMSNorm (融合)</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>_ZN5aiter37dynamic_per_token_scaled_quant_kernelItDB8_Li0EEE</t>
+          <t>_rms_norm_kernel</t>
         </is>
       </c>
       <c r="C30" t="n">
-        <v>505</v>
+        <v>0</v>
       </c>
       <c r="D30" t="n">
-        <v>14.1</v>
+        <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="F30" t="n">
-        <v>0</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>FP8 量化</t>
+          <t>RMSNorm (融合)</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>quant_fp8_blockwise_for_act_grad_kernel</t>
+          <t>_rmsnorm_kernel_large_m_small_n</t>
         </is>
       </c>
       <c r="C31" t="n">
-        <v>253</v>
+        <v>0</v>
       </c>
       <c r="D31" t="n">
-        <v>13.4</v>
+        <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>250</v>
+        <v>72</v>
       </c>
       <c r="F31" t="n">
-        <v>12.9</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>reduce (norm/softmax/sum)</t>
+          <t>RMSNorm (融合)</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>void at::native::reduce_kernel&lt;512, 1, at::native::ReduceOp&lt;</t>
+          <t>_rmsnorm_bwd_dg_reduce_triton</t>
         </is>
       </c>
       <c r="C32" t="n">
-        <v>289</v>
+        <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>9.800000000000001</v>
+        <v>0</v>
       </c>
       <c r="E32" t="n">
         <v>145</v>
       </c>
       <c r="F32" t="n">
-        <v>4.4</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>reduce (norm/softmax/sum)</t>
+          <t>dropout</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>void at::native::reduce_kernel&lt;512, 1, at::native::ReduceOp&lt;</t>
+          <t>void at::native::(anonymous namespace)::fused_dropout_kernel</t>
         </is>
       </c>
       <c r="C33" t="n">
-        <v>147</v>
+        <v>504</v>
       </c>
       <c r="D33" t="n">
-        <v>4.2</v>
+        <v>29.9</v>
       </c>
       <c r="E33" t="n">
-        <v>146</v>
+        <v>252</v>
       </c>
       <c r="F33" t="n">
-        <v>4.2</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>reduce (norm/softmax/sum)</t>
+          <t>FP8 量化</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>void at::native::reduce_kernel&lt;128, 4, at::native::ReduceOp&lt;</t>
+          <t>_ZN5aiter37dynamic_per_token_scaled_quant_kernelItDB8_Li0EEE</t>
         </is>
       </c>
       <c r="C34" t="n">
-        <v>0</v>
+        <v>505</v>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>14.1</v>
       </c>
       <c r="E34" t="n">
-        <v>72</v>
+        <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>2.2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>reduce (norm/softmax/sum)</t>
+          <t>FP8 量化</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>void at::native::(anonymous namespace)::cunn_SoftMaxForward&lt;</t>
+          <t>quant_fp8_blockwise_for_act_grad_kernel</t>
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1</v>
+        <v>253</v>
       </c>
       <c r="D35" t="n">
-        <v>1.3</v>
+        <v>13.4</v>
       </c>
       <c r="E35" t="n">
-        <v>1</v>
+        <v>253</v>
       </c>
       <c r="F35" t="n">
-        <v>1.3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="36">
@@ -1625,68 +1669,212 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>void at::native::(anonymous namespace)::cunn_SoftMaxBackward</t>
+          <t>void at::native::reduce_kernel&lt;512, 1, at::native::ReduceOp&lt;</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>1</v>
+        <v>289</v>
       </c>
       <c r="D36" t="n">
-        <v>1.1</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="E36" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>其他</t>
+          <t>reduce (norm/softmax/sum)</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>_ZN5aiter37dynamic_per_group_scaled_quant_kernelItDB8_Li32EE</t>
+          <t>void at::native::reduce_kernel&lt;512, 1, at::native::ReduceOp&lt;</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>505</v>
+        <v>147</v>
       </c>
       <c r="D37" t="n">
-        <v>9.300000000000001</v>
+        <v>4.2</v>
       </c>
       <c r="E37" t="n">
-        <v>253</v>
+        <v>2</v>
       </c>
       <c r="F37" t="n">
-        <v>4.7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>reduce (norm/softmax/sum)</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>void at::native::reduce_kernel&lt;128, 4, at::native::ReduceOp&lt;</t>
+        </is>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>72</v>
+      </c>
+      <c r="F38" t="n">
+        <v>2.2</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>reduce (norm/softmax/sum)</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>void at::native::(anonymous namespace)::cunn_SoftMaxForward&lt;</t>
+        </is>
+      </c>
+      <c r="C39" t="n">
+        <v>1</v>
+      </c>
+      <c r="D39" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E39" t="n">
+        <v>1</v>
+      </c>
+      <c r="F39" t="n">
+        <v>1.3</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>reduce (norm/softmax/sum)</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>void at::native::(anonymous namespace)::cunn_SoftMaxBackward</t>
+        </is>
+      </c>
+      <c r="C40" t="n">
+        <v>1</v>
+      </c>
+      <c r="D40" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="E40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>其他</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>_ZN5aiter37dynamic_per_group_scaled_quant_kernelItDB8_Li32EE</t>
+        </is>
+      </c>
+      <c r="C41" t="n">
+        <v>505</v>
+      </c>
+      <c r="D41" t="n">
+        <v>9.300000000000001</v>
+      </c>
+      <c r="E41" t="n">
+        <v>253</v>
+      </c>
+      <c r="F41" t="n">
+        <v>5.5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>其他</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
         <is>
           <t>bwd_preprocess</t>
         </is>
       </c>
-      <c r="C38" t="n">
+      <c r="C42" t="n">
         <v>36</v>
       </c>
-      <c r="D38" t="n">
+      <c r="D42" t="n">
         <v>0.7</v>
       </c>
-      <c r="E38" t="n">
-        <v>0</v>
-      </c>
-      <c r="F38" t="n">
-        <v>0</v>
+      <c r="E42" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>RoPE (融合)</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>_rope_kernel_sbhd_cached_fwd</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>72</v>
+      </c>
+      <c r="F43" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>RoPE (融合)</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>_rope_kernel_sbhd_cached_bwd</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>72</v>
+      </c>
+      <c r="F44" t="n">
+        <v>2.6</v>
       </c>
     </row>
   </sheetData>
@@ -1765,7 +1953,7 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>结论: param-storage 是给 70B 防 OOM 的; 8B 用 cache+shard_grad_op+no-ckpt+AITER attn 最快 (681ms)。</t>
+          <t>结论: param-storage 是给 70B 防 OOM 的; 8B 最快 = cache+shard_grad_op+no-ckpt+bpreshuffle+AITER attn+融合RMSNorm/RoPE (634ms)。</t>
         </is>
       </c>
     </row>
@@ -1795,14 +1983,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Qwen3-8B FSDP2 best + AITER attn(CK FMHA v3)— 每算子真实 shape + 实测/预估 latency (record_shapes)</t>
+          <t>Qwen3-8B FSDP2 best (AITER attn+融合RMSNorm/RoPE, 634ms)— 每算子真实 shape + 实测/预估 latency (record_shapes)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>chrome key_averages(group_by_input_shape), step15-17/3 | 实测 self-CUDA | FP8 GEMM 实测可达≈205 TFLOPS | 预估=FLOPs/可达吞吐</t>
+          <t>chrome key_averages(group_by_input_shape), step15-17/3 | 实测 self-CUDA | FP8 GEMM 实测可达≈209 TFLOPS | 预估=FLOPs/可达吞吐</t>
         </is>
       </c>
     </row>
@@ -1870,10 +2058,10 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>102.1</v>
+        <v>104.3</v>
       </c>
       <c r="F6" t="n">
-        <v>108.7</v>
+        <v>106.3</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -1901,10 +2089,10 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>100.1</v>
+        <v>100.5</v>
       </c>
       <c r="F7" t="n">
-        <v>108.7</v>
+        <v>106.3</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1924,18 +2112,18 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>9.83T</t>
+          <t>9.90T</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>62.8</v>
+        <v>47.8</v>
       </c>
       <c r="F8" t="n">
-        <v>48</v>
+        <v>47.3</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -1951,26 +2139,26 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2048×151936×4096</t>
+          <t>2048×1024×4096</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1</v>
+        <v>72</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2.55T</t>
+          <t>1.24T</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>11.6</v>
+        <v>13.7</v>
       </c>
       <c r="F9" t="n">
-        <v>12.4</v>
+        <v>5.9</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>lm_head·fwd</t>
+          <t>k/v_proj·fwd</t>
         </is>
       </c>
     </row>
@@ -1982,7 +2170,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2048×4096×151936</t>
+          <t>2048×151936×4096</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -1994,14 +2182,14 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>10.4</v>
+        <v>11.6</v>
       </c>
       <c r="F10" t="n">
-        <v>12.4</v>
+        <v>12.2</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>lm_head·dgrad</t>
+          <t>lm_head·fwd</t>
         </is>
       </c>
     </row>
@@ -2013,26 +2201,26 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2048×1024×4096</t>
+          <t>2048×4096×151936</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>72</v>
+        <v>1</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>1.24T</t>
+          <t>2.55T</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>7.6</v>
+        <v>10.4</v>
       </c>
       <c r="F11" t="n">
-        <v>6</v>
+        <v>12.2</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>k/v_proj·fwd</t>
+          <t>lm_head·dgrad</t>
         </is>
       </c>
     </row>
@@ -2048,15 +2236,15 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.20T</t>
+          <t>1.24T</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>7.6</v>
+        <v>7.8</v>
       </c>
       <c r="F12" t="n">
         <v>5.9</v>
@@ -2094,7 +2282,7 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>15.8</v>
+        <v>17.4</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -2127,7 +2315,7 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>41.7</v>
+        <v>41.6</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -2152,7 +2340,7 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1077</v>
+        <v>1296</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
@@ -2160,7 +2348,7 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>38</v>
+        <v>49.4</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -2185,7 +2373,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -2213,7 +2401,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
@@ -2221,7 +2409,7 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>23.7</v>
+        <v>26.8</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -2237,16 +2425,16 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>aten::cat (RoPE rotate_half)</t>
+          <t>aten::copy_ (contiguous/cast)</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>[[], []]</t>
+          <t>[[1, 32, 2048, 128], [1, 32, 2048, 128], []]</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>146</v>
+        <v>72</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -2254,32 +2442,27 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>7</v>
+        <v>4.4</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
           <t>-</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>可用 fused RoPE 省</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>aten::copy_ (contiguous/cast)</t>
+          <t>通信 all_gather</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>[[1, 2048, 4096], [1, 2048, 4096], []]</t>
+          <t>[]</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>833</v>
+        <v>37</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
@@ -2287,7 +2470,7 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>31.3</v>
+        <v>67.5</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -2298,7 +2481,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>通信 all_gather</t>
+          <t>通信 reduce_scatter</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2315,11 +2498,16 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>63.5</v>
+        <v>3.5</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
           <t>-</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>shard_grad_op 仅反向</t>
         </is>
       </c>
     </row>
@@ -2334,7 +2522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J74"/>
+  <dimension ref="A1:J69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2352,14 +2540,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Qwen3-8B FSDP2 best + AITER attention(CK FMHA v3)— 单算子明细(仅内层 GPU kernel)</t>
+          <t>Qwen3-8B FSDP2 best (AITER attn + 融合 RMSNorm + 融合 RoPE, 634ms)— 单算子明细(仅内层 GPU kernel)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>来源: chrome trace cat==kernel | step15-17/3 | 合计 696 ms/step(墙钟 ~681,对比 AOTriton 767)| attention=AITER CK FMHA v3(fmha_fwd/bwd_hd128_bf16_causal)| 预估=roofline: GEMM=max(FLOPs/206TFLOPS_FP8, bytes/HBM); attn=FLOPs/300TFLOPS(假设); 通信=bytes/300GB/s(假设); 访存=bytes/5.3TB/s(合并多shape的为近似≈)</t>
+          <t>来源: chrome trace cat==kernel | step15-17/3 | 合计 653 ms/step(墙钟 ~634;AOTriton baseline 767)| attention=AITER CK FMHA v3(fmha_fwd/bwd_hd128_bf16_causal)| 预估=roofline: GEMM=max(FLOPs/206TFLOPS_FP8, bytes/HBM); attn=FLOPs/300TFLOPS(假设); 通信=bytes/300GB/s(假设); 访存=bytes/5.3TB/s(合并多shape的为近似≈)</t>
         </is>
       </c>
     </row>
@@ -2433,7 +2621,7 @@
         <v>108</v>
       </c>
       <c r="E5" t="n">
-        <v>102.08</v>
+        <v>104.28</v>
       </c>
       <c r="F5" t="n">
         <v>108.08</v>
@@ -2445,11 +2633,11 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0.94x</t>
+          <t>0.96x</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>14.7</v>
+        <v>16</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -2475,7 +2663,7 @@
         <v>108</v>
       </c>
       <c r="E6" t="n">
-        <v>100.05</v>
+        <v>100.46</v>
       </c>
       <c r="F6" t="n">
         <v>108.08</v>
@@ -2491,7 +2679,7 @@
         </is>
       </c>
       <c r="I6" t="n">
-        <v>14.4</v>
+        <v>15.4</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -2514,10 +2702,10 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E7" t="n">
-        <v>66.26000000000001</v>
+        <v>71.11</v>
       </c>
       <c r="F7" t="n">
         <v>50.07</v>
@@ -2529,11 +2717,11 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>1.32x</t>
+          <t>1.42x</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>9.5</v>
+        <v>10.9</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -2556,13 +2744,13 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E8" t="n">
-        <v>62.8</v>
+        <v>47.84</v>
       </c>
       <c r="F8" t="n">
-        <v>47.7</v>
+        <v>48.04</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -2571,11 +2759,11 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>1.32x</t>
+          <t>1.00x</t>
         </is>
       </c>
       <c r="I8" t="n">
-        <v>9</v>
+        <v>7.3</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -2601,7 +2789,7 @@
         <v>36</v>
       </c>
       <c r="E9" t="n">
-        <v>37.09</v>
+        <v>37.08</v>
       </c>
       <c r="F9" t="n">
         <v>10.31</v>
@@ -2617,7 +2805,7 @@
         </is>
       </c>
       <c r="I9" t="n">
-        <v>5.3</v>
+        <v>5.7</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -2631,22 +2819,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">void at::native::elementwise_kernel_manual_unroll&lt;128, 8, </t>
+          <t>_rmsnorm_bwd_triton</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>[2048,4096]</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>577</v>
+        <v>145</v>
       </c>
       <c r="E10" t="n">
-        <v>21.68</v>
+        <v>36.35</v>
       </c>
       <c r="F10" t="n">
-        <v>3.65</v>
+        <v>0.92</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -2655,15 +2843,15 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>5.93x</t>
+          <t>39.60x</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>3.1</v>
+        <v>5.6</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>融合 RMSNorm 反向(dX+dW)</t>
         </is>
       </c>
     </row>
@@ -2682,13 +2870,13 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>858</v>
+        <v>755</v>
       </c>
       <c r="E11" t="n">
-        <v>18.69</v>
+        <v>18</v>
       </c>
       <c r="F11" t="n">
-        <v>5.43</v>
+        <v>4.78</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -2697,11 +2885,11 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>3.44x</t>
+          <t>3.77x</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>2.7</v>
+        <v>2.8</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -2715,22 +2903,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">void at::native::elementwise_kernel_manual_unroll&lt;128, 4, </t>
+          <t>void at::native::(anonymous namespace)::fused_dropout_kern</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>[1,2048,4096]</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>291</v>
+        <v>252</v>
       </c>
       <c r="E12" t="n">
-        <v>18.09</v>
+        <v>17.4</v>
       </c>
       <c r="F12" t="n">
-        <v>1.84</v>
+        <v>1.6</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -2739,15 +2927,15 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>9.82x</t>
+          <t>10.90x</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>2.6</v>
+        <v>2.7</v>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>dropout 前向</t>
         </is>
       </c>
     </row>
@@ -2769,7 +2957,7 @@
         <v>36</v>
       </c>
       <c r="E13" t="n">
-        <v>15.84</v>
+        <v>17.36</v>
       </c>
       <c r="F13" t="n">
         <v>4.12</v>
@@ -2781,11 +2969,11 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>3.84x</t>
+          <t>4.21x</t>
         </is>
       </c>
       <c r="I13" t="n">
-        <v>2.3</v>
+        <v>2.7</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -2808,13 +2996,13 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="E14" t="n">
-        <v>14.37</v>
+        <v>15.02</v>
       </c>
       <c r="F14" t="n">
-        <v>1.03</v>
+        <v>1.04</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -2823,11 +3011,11 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>13.98x</t>
+          <t>14.47x</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>2.1</v>
+        <v>2.3</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -2841,39 +3029,39 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>void at::native::(anonymous namespace)::fused_dropout_kern</t>
+          <t>ck::kernel_gemm_xdl_cshuffle_v3_multi_d_blockscale</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>[1,2048,4096]</t>
+          <t>2048×1024×4096</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>252</v>
+        <v>72</v>
       </c>
       <c r="E15" t="n">
-        <v>14.12</v>
+        <v>13.67</v>
       </c>
       <c r="F15" t="n">
-        <v>1.6</v>
+        <v>6</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>memory</t>
+          <t>compute</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>8.85x</t>
+          <t>2.28x</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>2</v>
+        <v>2.1</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>dropout 前向</t>
+          <t>FP8 blockwise2d GEMM(内层 CK kernel)</t>
         </is>
       </c>
     </row>
@@ -2883,22 +3071,22 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">void at::native::elementwise_kernel_manual_unroll&lt;128, 4, </t>
+          <t>at::native::detail::split_with_sizes_copy_out_contiguous_n</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>[8,24269856]</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>362</v>
+        <v>37</v>
       </c>
       <c r="E16" t="n">
-        <v>13.32</v>
+        <v>13.38</v>
       </c>
       <c r="F16" t="n">
-        <v>2.29</v>
+        <v>5.42</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -2907,15 +3095,15 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>5.81x</t>
+          <t>2.47x</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>FSDP all-gather 解包(8卡分片)</t>
         </is>
       </c>
     </row>
@@ -2925,22 +3113,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>at::native::detail::split_with_sizes_copy_out_contiguous_n</t>
+          <t>quant_fp8_blockwise_for_act_grad_kernel</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>[8,24269856]</t>
+          <t>[2048,4096]/[2048,12288]</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>37</v>
+        <v>253</v>
       </c>
       <c r="E17" t="n">
-        <v>13.29</v>
+        <v>13.01</v>
       </c>
       <c r="F17" t="n">
-        <v>5.42</v>
+        <v>1.6</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -2949,15 +3137,15 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>2.45x</t>
+          <t>8.13x</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>FSDP all-gather 解包(8卡分片)</t>
+          <t>梯度量化→fp8(1×128)</t>
         </is>
       </c>
     </row>
@@ -2967,22 +3155,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>quant_fp8_blockwise_for_act_grad_kernel</t>
+          <t xml:space="preserve">void at::native::elementwise_kernel_manual_unroll&lt;128, 8, </t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>[2048,4096]/[2048,12288]</t>
+          <t>[1,2048,4096]/[1,2048,12288]</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>250</v>
+        <v>324</v>
       </c>
       <c r="E18" t="n">
-        <v>12.94</v>
+        <v>12.23</v>
       </c>
       <c r="F18" t="n">
-        <v>1.58</v>
+        <v>2.05</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -2991,7 +3179,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>8.18x</t>
+          <t>5.96x</t>
         </is>
       </c>
       <c r="I18" t="n">
@@ -2999,7 +3187,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>梯度量化→fp8(1×128)</t>
+          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
         </is>
       </c>
     </row>
@@ -3021,7 +3209,7 @@
         <v>1</v>
       </c>
       <c r="E19" t="n">
-        <v>11.57</v>
+        <v>11.56</v>
       </c>
       <c r="F19" t="n">
         <v>12.37</v>
@@ -3037,7 +3225,7 @@
         </is>
       </c>
       <c r="I19" t="n">
-        <v>1.7</v>
+        <v>1.8</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -3051,39 +3239,39 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ck::kernel_gemm_xdl_cshuffle_v3_multi_d_blockscale</t>
+          <t>void at::native::vectorized_elementwise_kernel&lt;8, at::nati</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2048×4096×151936</t>
+          <t>[1,2048,4096]/[1,2048,12288]</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1</v>
+        <v>505</v>
       </c>
       <c r="E20" t="n">
-        <v>10.44</v>
+        <v>10.8</v>
       </c>
       <c r="F20" t="n">
-        <v>12.37</v>
+        <v>3.2</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>compute</t>
+          <t>memory</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>0.84x</t>
+          <t>3.38x</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>FP8 blockwise2d GEMM(内层 CK kernel)</t>
+          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
         </is>
       </c>
     </row>
@@ -3093,39 +3281,39 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>void at::native::vectorized_elementwise_kernel&lt;8, at::nati</t>
+          <t>ck::kernel_gemm_xdl_cshuffle_v3_multi_d_blockscale</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>2048×4096×151936</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>505</v>
+        <v>1</v>
       </c>
       <c r="E21" t="n">
-        <v>10.15</v>
+        <v>10.43</v>
       </c>
       <c r="F21" t="n">
-        <v>3.2</v>
+        <v>12.37</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>memory</t>
+          <t>compute</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>3.17x</t>
+          <t>0.84x</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>FP8 blockwise2d GEMM(内层 CK kernel)</t>
         </is>
       </c>
     </row>
@@ -3147,7 +3335,7 @@
         <v>108</v>
       </c>
       <c r="E22" t="n">
-        <v>8.970000000000001</v>
+        <v>10.19</v>
       </c>
       <c r="F22" t="n">
         <v>1.03</v>
@@ -3159,11 +3347,11 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>8.66x</t>
+          <t>9.85x</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>1.3</v>
+        <v>1.6</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -3177,39 +3365,39 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ck::kernel_gemm_xdl_cshuffle_v3_multi_d_blockscale</t>
+          <t>Cijk_* (hipBLASLt bf16 GEMM)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2048×1024×4096</t>
+          <t>2048×16×4096</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>72</v>
+        <v>324</v>
       </c>
       <c r="E23" t="n">
-        <v>7.65</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="F23" t="n">
-        <v>6</v>
+        <v>1.04</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>compute</t>
+          <t>memory</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>1.27x</t>
+          <t>7.99x</t>
         </is>
       </c>
       <c r="I23" t="n">
-        <v>1.1</v>
+        <v>1.3</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>FP8 blockwise2d GEMM(内层 CK kernel)</t>
+          <t>LoRA A/B/wgrad</t>
         </is>
       </c>
     </row>
@@ -3228,13 +3416,13 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E24" t="n">
-        <v>7.56</v>
+        <v>7.79</v>
       </c>
       <c r="F24" t="n">
-        <v>5.84</v>
+        <v>6</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -3247,7 +3435,7 @@
         </is>
       </c>
       <c r="I24" t="n">
-        <v>1.1</v>
+        <v>1.2</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -3261,22 +3449,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Cijk_* (hipBLASLt bf16 GEMM)</t>
+          <t>void at::native::vectorized_elementwise_kernel&lt;8, at::nati</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>2048×16×4096</t>
+          <t>[1,2048,4096]/[1,2048,12288]</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>324</v>
+        <v>252</v>
       </c>
       <c r="E25" t="n">
-        <v>7.19</v>
+        <v>6.24</v>
       </c>
       <c r="F25" t="n">
-        <v>1.04</v>
+        <v>1.6</v>
       </c>
       <c r="G25" t="inlineStr">
         <is>
@@ -3285,7 +3473,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>6.93x</t>
+          <t>3.91x</t>
         </is>
       </c>
       <c r="I25" t="n">
@@ -3293,7 +3481,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>LoRA A/B/wgrad</t>
+          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
         </is>
       </c>
     </row>
@@ -3303,22 +3491,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>void at::native::(anonymous namespace)::CatArrayBatchedCop</t>
+          <t>_ZN5aiter37dynamic_per_group_scaled_quant_kernelItDB8_Li32</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>[1,32,2048,128]</t>
+          <t>[2048,4096]/[2048,12288]</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>144</v>
+        <v>253</v>
       </c>
       <c r="E26" t="n">
-        <v>7.01</v>
+        <v>5.48</v>
       </c>
       <c r="F26" t="n">
-        <v>0.91</v>
+        <v>1.6</v>
       </c>
       <c r="G26" t="inlineStr">
         <is>
@@ -3327,15 +3515,15 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>7.69x</t>
+          <t>3.42x</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>RoPE rotate_half cat</t>
+          <t>激活量化→fp8</t>
         </is>
       </c>
     </row>
@@ -3345,7 +3533,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">void at::native::elementwise_kernel_manual_unroll&lt;128, 4, </t>
+          <t>void at::native::vectorized_elementwise_kernel&lt;8, at::nati</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3354,13 +3542,13 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>144</v>
+        <v>108</v>
       </c>
       <c r="E27" t="n">
-        <v>6.91</v>
+        <v>5.1</v>
       </c>
       <c r="F27" t="n">
-        <v>0.91</v>
+        <v>0.68</v>
       </c>
       <c r="G27" t="inlineStr">
         <is>
@@ -3369,11 +3557,11 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>7.58x</t>
+          <t>7.46x</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -3387,22 +3575,24 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">void at::native::elementwise_kernel_manual_unroll&lt;128, 8, </t>
+          <t>void at::native::(anonymous namespace)::multi_tensor_apply</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>LoRA ~44M(多小张量)</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>252</v>
+        <v>80</v>
       </c>
       <c r="E28" t="n">
-        <v>6.66</v>
-      </c>
-      <c r="F28" t="n">
-        <v>1.6</v>
+        <v>4.92</v>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -3411,15 +3601,15 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>4.17x</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>AdamW foreach(launch-bound)</t>
         </is>
       </c>
     </row>
@@ -3429,7 +3619,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>void at::native::vectorized_elementwise_kernel&lt;4, at::nati</t>
+          <t>void at::native::vectorized_elementwise_kernel&lt;8, at::nati</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3438,13 +3628,13 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>360</v>
+        <v>36</v>
       </c>
       <c r="E29" t="n">
-        <v>6.08</v>
+        <v>4.53</v>
       </c>
       <c r="F29" t="n">
-        <v>2.28</v>
+        <v>0.23</v>
       </c>
       <c r="G29" t="inlineStr">
         <is>
@@ -3453,11 +3643,11 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>2.67x</t>
+          <t>19.88x</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>0.9</v>
+        <v>0.7</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -3471,7 +3661,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>void at::native::vectorized_elementwise_kernel&lt;4, at::nati</t>
+          <t>void at::native::vectorized_elementwise_kernel&lt;8, at::nati</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3480,13 +3670,13 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>328</v>
+        <v>36</v>
       </c>
       <c r="E30" t="n">
-        <v>6.05</v>
+        <v>4.23</v>
       </c>
       <c r="F30" t="n">
-        <v>2.08</v>
+        <v>0.23</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -3495,11 +3685,11 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>2.91x</t>
+          <t>18.57x</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="J30" t="inlineStr">
         <is>
@@ -3513,22 +3703,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>void at::native::vectorized_elementwise_kernel&lt;8, at::nati</t>
+          <t>Cijk_* (hipBLASLt bf16 GEMM)</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>16×4096×2048</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>249</v>
+        <v>216</v>
       </c>
       <c r="E31" t="n">
-        <v>6.01</v>
+        <v>4.15</v>
       </c>
       <c r="F31" t="n">
-        <v>1.58</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -3537,15 +3727,15 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>3.81x</t>
+          <t>5.99x</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>LoRA A/B/wgrad</t>
         </is>
       </c>
     </row>
@@ -3555,24 +3745,22 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>void at::native::(anonymous namespace)::multi_tensor_apply</t>
+          <t xml:space="preserve">void at::native::elementwise_kernel_manual_unroll&lt;128, 4, </t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LoRA ~44M(多小张量)</t>
+          <t>[1,2048,4096]/[1,2048,12288]</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>80</v>
+        <v>506</v>
       </c>
       <c r="E32" t="n">
-        <v>5.91</v>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+        <v>3.87</v>
+      </c>
+      <c r="F32" t="n">
+        <v>3.2</v>
       </c>
       <c r="G32" t="inlineStr">
         <is>
@@ -3581,15 +3769,15 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>1.21x</t>
         </is>
       </c>
       <c r="I32" t="n">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>AdamW foreach(launch-bound)</t>
+          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
         </is>
       </c>
     </row>
@@ -3599,22 +3787,22 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>void at::native::vectorized_elementwise_kernel&lt;8, at::nati</t>
+          <t>Cijk_* (hipBLASLt bf16 GEMM)</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>2048×16×12288</t>
         </is>
       </c>
       <c r="D33" t="n">
         <v>108</v>
       </c>
       <c r="E33" t="n">
-        <v>4.88</v>
+        <v>3.27</v>
       </c>
       <c r="F33" t="n">
-        <v>0.68</v>
+        <v>1.03</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -3623,15 +3811,15 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>7.14x</t>
+          <t>3.16x</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>LoRA A/B/wgrad</t>
         </is>
       </c>
     </row>
@@ -3641,22 +3829,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>_ZN5aiter37dynamic_per_group_scaled_quant_kernelItDB8_Li32</t>
+          <t>Cijk_* (hipBLASLt bf16 GEMM)</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>[2048,4096]/[2048,12288]</t>
+          <t>12288×16×2048</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>253</v>
+        <v>72</v>
       </c>
       <c r="E34" t="n">
-        <v>4.72</v>
+        <v>3.24</v>
       </c>
       <c r="F34" t="n">
-        <v>1.6</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -3665,15 +3853,15 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>2.95x</t>
+          <t>4.70x</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>0.7</v>
+        <v>0.5</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>激活量化→fp8</t>
+          <t>LoRA A/B/wgrad</t>
         </is>
       </c>
     </row>
@@ -3683,22 +3871,22 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>void at::native::vectorized_elementwise_kernel&lt;8, at::nati</t>
+          <t>_rms_norm_kernel</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>[2048,4096]</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>36</v>
+        <v>73</v>
       </c>
       <c r="E35" t="n">
-        <v>4.53</v>
+        <v>2.87</v>
       </c>
       <c r="F35" t="n">
-        <v>0.23</v>
+        <v>0.46</v>
       </c>
       <c r="G35" t="inlineStr">
         <is>
@@ -3707,15 +3895,15 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>19.89x</t>
+          <t>6.21x</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>0.7</v>
+        <v>0.4</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>融合 RMSNorm 前向</t>
         </is>
       </c>
     </row>
@@ -3725,22 +3913,22 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">void at::native::elementwise_kernel_manual_unroll&lt;128, 8, </t>
+          <t>aiter::fmha_bwd_hd128_dq_convert_bf16_rtna</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>[1,32,2048,128]</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>108</v>
+        <v>36</v>
       </c>
       <c r="E36" t="n">
-        <v>4.5</v>
+        <v>2.77</v>
       </c>
       <c r="F36" t="n">
-        <v>0.68</v>
+        <v>0.23</v>
       </c>
       <c r="G36" t="inlineStr">
         <is>
@@ -3749,15 +3937,15 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>6.58x</t>
+          <t>12.16x</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>CK FMHA v3 反向: dq 转 bf16(访存)</t>
         </is>
       </c>
     </row>
@@ -3767,22 +3955,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>void at::native::reduce_kernel&lt;512, 1, at::native::ReduceO</t>
+          <t>_rope_kernel_sbhd_cached_fwd</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>[2048,4096]</t>
+          <t>[1,32,2048,128]</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>145</v>
+        <v>72</v>
       </c>
       <c r="E37" t="n">
-        <v>4.36</v>
+        <v>2.72</v>
       </c>
       <c r="F37" t="n">
-        <v>0.92</v>
+        <v>0.46</v>
       </c>
       <c r="G37" t="inlineStr">
         <is>
@@ -3791,15 +3979,15 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>4.75x</t>
+          <t>5.97x</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>reduce(sum/mean/softmax)</t>
+          <t>融合 RoPE(AITER fwd/bwd)</t>
         </is>
       </c>
     </row>
@@ -3809,22 +3997,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Cijk_* (hipBLASLt bf16 GEMM)</t>
+          <t>_rope_kernel_sbhd_cached_bwd</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>16×4096×2048</t>
+          <t>[1,32,2048,128]</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>216</v>
+        <v>72</v>
       </c>
       <c r="E38" t="n">
-        <v>4.22</v>
+        <v>2.64</v>
       </c>
       <c r="F38" t="n">
-        <v>0.6899999999999999</v>
+        <v>0.46</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -3833,15 +4021,15 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>6.10x</t>
+          <t>5.79x</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>LoRA A/B/wgrad</t>
+          <t>融合 RoPE(AITER fwd/bwd)</t>
         </is>
       </c>
     </row>
@@ -3851,22 +4039,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>void at::native::reduce_kernel&lt;512, 1, at::native::ReduceO</t>
+          <t>Cijk_* (hipBLASLt bf16 GEMM)</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>[2048,4096]</t>
+          <t>4096×16×2048</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>146</v>
+        <v>108</v>
       </c>
       <c r="E39" t="n">
-        <v>4.2</v>
+        <v>2.64</v>
       </c>
       <c r="F39" t="n">
-        <v>0.92</v>
+        <v>0.35</v>
       </c>
       <c r="G39" t="inlineStr">
         <is>
@@ -3875,15 +4063,15 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>4.54x</t>
+          <t>7.63x</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>reduce(sum/mean/softmax)</t>
+          <t>LoRA A/B/wgrad</t>
         </is>
       </c>
     </row>
@@ -3893,22 +4081,22 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>void at::native::vectorized_elementwise_kernel&lt;8, at::nati</t>
+          <t>Cijk_* (hipBLASLt bf16 GEMM)</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>16×12288×2048</t>
         </is>
       </c>
       <c r="D40" t="n">
         <v>36</v>
       </c>
       <c r="E40" t="n">
-        <v>4.19</v>
+        <v>2.62</v>
       </c>
       <c r="F40" t="n">
-        <v>0.23</v>
+        <v>0.34</v>
       </c>
       <c r="G40" t="inlineStr">
         <is>
@@ -3917,15 +4105,15 @@
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>18.40x</t>
+          <t>7.60x</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>LoRA A/B/wgrad</t>
         </is>
       </c>
     </row>
@@ -3935,22 +4123,22 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Memcpy DtoD (Device -&gt; Device)</t>
+          <t>void at::native::(anonymous namespace)::CatArrayBatchedCop</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>[1,2048,4096]</t>
+          <t>[1,32,2048,128]</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>188</v>
+        <v>72</v>
       </c>
       <c r="E41" t="n">
-        <v>4.11</v>
+        <v>2.39</v>
       </c>
       <c r="F41" t="n">
-        <v>1.19</v>
+        <v>0.46</v>
       </c>
       <c r="G41" t="inlineStr">
         <is>
@@ -3959,15 +4147,15 @@
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>3.45x</t>
+          <t>5.25x</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>0.6</v>
+        <v>0.4</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>设备内存拷贝</t>
+          <t>RoPE rotate_half cat</t>
         </is>
       </c>
     </row>
@@ -3977,22 +4165,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">void at::native::elementwise_kernel_manual_unroll&lt;128, 4, </t>
+          <t>void at::native::reduce_kernel&lt;128, 4, at::native::ReduceO</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>[2048,4096]</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>503</v>
+        <v>72</v>
       </c>
       <c r="E42" t="n">
-        <v>3.65</v>
+        <v>2.17</v>
       </c>
       <c r="F42" t="n">
-        <v>3.18</v>
+        <v>0.46</v>
       </c>
       <c r="G42" t="inlineStr">
         <is>
@@ -4001,15 +4189,15 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>1.14x</t>
+          <t>4.77x</t>
         </is>
       </c>
       <c r="I42" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>reduce(sum/mean/softmax)</t>
         </is>
       </c>
     </row>
@@ -4019,22 +4207,22 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>void at::native::vectorized_elementwise_kernel&lt;4, at::nati</t>
+          <t>_rmsnorm_kernel_large_m_small_n</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>[2048,4096]</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>290</v>
+        <v>72</v>
       </c>
       <c r="E43" t="n">
-        <v>3.36</v>
+        <v>2.14</v>
       </c>
       <c r="F43" t="n">
-        <v>1.84</v>
+        <v>0.46</v>
       </c>
       <c r="G43" t="inlineStr">
         <is>
@@ -4043,15 +4231,15 @@
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>1.83x</t>
+          <t>4.68x</t>
         </is>
       </c>
       <c r="I43" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>融合 RMSNorm 前向</t>
         </is>
       </c>
     </row>
@@ -4061,22 +4249,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Cijk_* (hipBLASLt bf16 GEMM)</t>
+          <t>aiter::fmha_bwd_hd128_odo_bf16</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>2048×16×12288</t>
+          <t>[1,32,2048,128]</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>108</v>
+        <v>36</v>
       </c>
       <c r="E44" t="n">
-        <v>3.26</v>
+        <v>1.78</v>
       </c>
       <c r="F44" t="n">
-        <v>1.03</v>
+        <v>0.23</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -4085,15 +4273,15 @@
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>3.15x</t>
+          <t>7.83x</t>
         </is>
       </c>
       <c r="I44" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>LoRA A/B/wgrad</t>
+          <t>CK FMHA v3 反向: O·dO 预处理(访存)</t>
         </is>
       </c>
     </row>
@@ -4103,22 +4291,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>void at::native::vectorized_elementwise_kernel&lt;4, at::nati</t>
+          <t>void at::native::(anonymous namespace)::cunn_SoftMaxForwar</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>[2048,151936]</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>145</v>
+        <v>1</v>
       </c>
       <c r="E45" t="n">
-        <v>3.17</v>
+        <v>1.28</v>
       </c>
       <c r="F45" t="n">
-        <v>0.92</v>
+        <v>0.23</v>
       </c>
       <c r="G45" t="inlineStr">
         <is>
@@ -4127,15 +4315,15 @@
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>3.45x</t>
+          <t>5.45x</t>
         </is>
       </c>
       <c r="I45" t="n">
-        <v>0.5</v>
+        <v>0.2</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>loss/softmax(lm_head logits)</t>
         </is>
       </c>
     </row>
@@ -4145,22 +4333,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">void at::native::elementwise_kernel_manual_unroll&lt;128, 8, </t>
+          <t>void at::native::(anonymous namespace)::cunn_SoftMaxBackwa</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>[2048,151936]</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>144</v>
+        <v>1</v>
       </c>
       <c r="E46" t="n">
-        <v>2.83</v>
+        <v>1.06</v>
       </c>
       <c r="F46" t="n">
-        <v>0.91</v>
+        <v>0.23</v>
       </c>
       <c r="G46" t="inlineStr">
         <is>
@@ -4169,15 +4357,15 @@
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>3.11x</t>
+          <t>4.53x</t>
         </is>
       </c>
       <c r="I46" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>loss/softmax(lm_head logits)</t>
         </is>
       </c>
     </row>
@@ -4187,22 +4375,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>aiter::fmha_bwd_hd128_dq_convert_bf16_rtna</t>
+          <t>_rmsnorm_bwd_dg_reduce_triton</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>[1,32,2048,128]</t>
+          <t>[2048,4096]</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>36</v>
+        <v>145</v>
       </c>
       <c r="E47" t="n">
-        <v>2.79</v>
+        <v>0.84</v>
       </c>
       <c r="F47" t="n">
-        <v>0.23</v>
+        <v>0.92</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -4211,15 +4399,15 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>12.25x</t>
+          <t>0.92x</t>
         </is>
       </c>
       <c r="I47" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>CK FMHA v3 反向: dq 转 bf16(访存)</t>
+          <t>融合 RMSNorm 反向(dX+dW)</t>
         </is>
       </c>
     </row>
@@ -4229,7 +4417,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">void at::native::elementwise_kernel_manual_unroll&lt;128, 4, </t>
+          <t>void at::native::vectorized_elementwise_kernel&lt;4, at::nati</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -4238,13 +4426,13 @@
         </is>
       </c>
       <c r="D48" t="n">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E48" t="n">
-        <v>2.66</v>
+        <v>0.8</v>
       </c>
       <c r="F48" t="n">
-        <v>0.46</v>
+        <v>0.47</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -4253,11 +4441,11 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>5.83x</t>
+          <t>1.72x</t>
         </is>
       </c>
       <c r="I48" t="n">
-        <v>0.4</v>
+        <v>0.1</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -4271,7 +4459,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>void at::native::vectorized_elementwise_kernel&lt;4, at::nati</t>
+          <t>void at::native::vectorized_elementwise_kernel&lt;8, at::nati</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -4280,13 +4468,13 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>72</v>
+        <v>41</v>
       </c>
       <c r="E49" t="n">
-        <v>2.32</v>
+        <v>0.75</v>
       </c>
       <c r="F49" t="n">
-        <v>0.46</v>
+        <v>0.26</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -4295,11 +4483,11 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>5.09x</t>
+          <t>2.89x</t>
         </is>
       </c>
       <c r="I49" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
@@ -4313,22 +4501,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>void at::native::reduce_kernel&lt;128, 4, at::native::ReduceO</t>
+          <t>Memcpy HtoD (Host -&gt; Device)</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>[2048,4096]</t>
+          <t>[1,2048,4096]</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>72</v>
+        <v>37</v>
       </c>
       <c r="E50" t="n">
-        <v>2.18</v>
+        <v>0.53</v>
       </c>
       <c r="F50" t="n">
-        <v>0.46</v>
+        <v>0.23</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -4337,15 +4525,15 @@
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>4.78x</t>
+          <t>2.26x</t>
         </is>
       </c>
       <c r="I50" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>reduce(sum/mean/softmax)</t>
+          <t>设备内存拷贝</t>
         </is>
       </c>
     </row>
@@ -4355,22 +4543,22 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>void at::native::vectorized_elementwise_kernel&lt;8, at::nati</t>
+          <t>void at::native::detail::chunk_cat_cuda_kernel&lt;float, c10:</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>[1,2048,4096]</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>185</v>
+        <v>37</v>
       </c>
       <c r="E51" t="n">
-        <v>1.98</v>
+        <v>0.41</v>
       </c>
       <c r="F51" t="n">
-        <v>1.17</v>
+        <v>0.23</v>
       </c>
       <c r="G51" t="inlineStr">
         <is>
@@ -4379,15 +4567,15 @@
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>1.69x</t>
+          <t>1.74x</t>
         </is>
       </c>
       <c r="I51" t="n">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>chunk/cat(RoPE/concat)</t>
         </is>
       </c>
     </row>
@@ -4397,22 +4585,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>aiter::fmha_bwd_hd128_odo_bf16</t>
+          <t>Memcpy DtoD (Device -&gt; Device)</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>[1,32,2048,128]</t>
+          <t>[1,2048,4096]</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="E52" t="n">
-        <v>1.78</v>
+        <v>0.27</v>
       </c>
       <c r="F52" t="n">
-        <v>0.23</v>
+        <v>0.28</v>
       </c>
       <c r="G52" t="inlineStr">
         <is>
@@ -4421,15 +4609,15 @@
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>7.80x</t>
+          <t>0.94x</t>
         </is>
       </c>
       <c r="I52" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>CK FMHA v3 反向: O·dO 预处理(访存)</t>
+          <t>设备内存拷贝</t>
         </is>
       </c>
     </row>
@@ -4439,22 +4627,22 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>void at::native::(anonymous namespace)::cunn_SoftMaxForwar</t>
+          <t>void at::native::vectorized_elementwise_kernel&lt;4, at::nati</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>[2048,151936]</t>
+          <t>[1,2048,4096]/[1,2048,12288]</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>1</v>
+        <v>40</v>
       </c>
       <c r="E53" t="n">
-        <v>1.29</v>
+        <v>0.23</v>
       </c>
       <c r="F53" t="n">
-        <v>0.23</v>
+        <v>0.25</v>
       </c>
       <c r="G53" t="inlineStr">
         <is>
@@ -4463,15 +4651,15 @@
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>5.49x</t>
+          <t>0.91x</t>
         </is>
       </c>
       <c r="I53" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>loss/softmax(lm_head logits)</t>
+          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
         </is>
       </c>
     </row>
@@ -4481,22 +4669,24 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>void at::native::(anonymous namespace)::cunn_SoftMaxBackwa</t>
+          <t>void at::native::(anonymous namespace)::multi_tensor_apply</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>[2048,151936]</t>
+          <t>LoRA ~44M(多小张量)</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E54" t="n">
-        <v>1.06</v>
-      </c>
-      <c r="F54" t="n">
-        <v>0.23</v>
+        <v>0.18</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
@@ -4505,15 +4695,15 @@
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>4.53x</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I54" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>loss/softmax(lm_head logits)</t>
+          <t>AdamW foreach(launch-bound)</t>
         </is>
       </c>
     </row>
@@ -4523,22 +4713,24 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>void at::native::vectorized_elementwise_kernel&lt;4, at::nati</t>
+          <t>void at::native::(anonymous namespace)::multi_tensor_apply</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>LoRA ~44M(多小张量)</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>145</v>
+        <v>12</v>
       </c>
       <c r="E55" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="F55" t="n">
-        <v>0.92</v>
+        <v>0.15</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
@@ -4547,15 +4739,15 @@
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>1.15x</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I55" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>AdamW foreach(launch-bound)</t>
         </is>
       </c>
     </row>
@@ -4565,22 +4757,24 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>void at::native::vectorized_elementwise_kernel&lt;4, at::nati</t>
+          <t>void at::native::(anonymous namespace)::multi_tensor_apply</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>LoRA ~44M(多小张量)</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>145</v>
+        <v>11</v>
       </c>
       <c r="E56" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="F56" t="n">
-        <v>0.92</v>
+        <v>0.13</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
@@ -4589,15 +4783,15 @@
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1.07x</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I56" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>AdamW foreach(launch-bound)</t>
         </is>
       </c>
     </row>
@@ -4607,22 +4801,24 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>void at::native::vectorized_elementwise_kernel&lt;4, at::nati</t>
+          <t>void at::native::(anonymous namespace)::multi_tensor_apply</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>LoRA ~44M(多小张量)</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>144</v>
+        <v>14</v>
       </c>
       <c r="E57" t="n">
-        <v>0.86</v>
-      </c>
-      <c r="F57" t="n">
-        <v>0.91</v>
+        <v>0.13</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -4631,15 +4827,15 @@
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>0.95x</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I57" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
+          <t>AdamW foreach(launch-bound)</t>
         </is>
       </c>
     </row>
@@ -4649,22 +4845,24 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>void at::native::vectorized_elementwise_kernel&lt;4, at::nati</t>
+          <t>void at::native::(anonymous namespace)::multi_tensor_apply</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>[1,2048,4096]/[1,2048,12288]</t>
+          <t>LoRA ~44M(多小张量)</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>74</v>
+        <v>11</v>
       </c>
       <c r="E58" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="F58" t="n">
-        <v>0.47</v>
+        <v>0.12</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
       </c>
       <c r="G58" t="inlineStr">
         <is>
@@ -4673,344 +4871,128 @@
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>1.75x</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I58" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>elementwise(norm/residual/swiglu/scale/cast/copy)</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="n">
-        <v>55</v>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Memcpy HtoD (Host -&gt; Device)</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>[1,2048,4096]</t>
-        </is>
-      </c>
-      <c r="D59" t="n">
-        <v>37</v>
-      </c>
-      <c r="E59" t="n">
-        <v>0.53</v>
-      </c>
-      <c r="F59" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>memory</t>
-        </is>
-      </c>
-      <c r="H59" t="inlineStr">
-        <is>
-          <t>2.26x</t>
-        </is>
-      </c>
-      <c r="I59" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="J59" t="inlineStr">
-        <is>
-          <t>设备内存拷贝</t>
+          <t>AdamW foreach(launch-bound)</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" t="n">
-        <v>56</v>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>void at::native::detail::chunk_cat_cuda_kernel&lt;float, c10:</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>[1,2048,4096]</t>
-        </is>
-      </c>
-      <c r="D60" t="n">
-        <v>36</v>
-      </c>
-      <c r="E60" t="n">
-        <v>0.42</v>
-      </c>
-      <c r="F60" t="n">
-        <v>0.23</v>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>memory</t>
-        </is>
-      </c>
-      <c r="H60" t="inlineStr">
-        <is>
-          <t>1.84x</t>
-        </is>
-      </c>
-      <c r="I60" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="J60" t="inlineStr">
-        <is>
-          <t>chunk/cat(RoPE/concat)</t>
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>shape 含义图例</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" t="n">
-        <v>57</v>
+      <c r="A61" s="3" t="inlineStr">
+        <is>
+          <t>FP8 GEMM (ck::kernel_gemm)</t>
+        </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>void at::native::(anonymous namespace)::multi_tensor_apply</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>LoRA ~44M(多小张量)</t>
-        </is>
-      </c>
-      <c r="D61" t="n">
-        <v>11</v>
-      </c>
-      <c r="E61" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="F61" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>memory</t>
-        </is>
-      </c>
-      <c r="H61" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I61" t="n">
-        <v>0</v>
-      </c>
-      <c r="J61" t="inlineStr">
-        <is>
-          <t>AdamW foreach(launch-bound)</t>
+          <t>shape=M×N×K (M=2048,N/K∈{4096,12288,1024,151936});实参=[激活X(M,K)fp8, 权重W(N,K)fp8, 激活scale(M,K/128), 权重scale(N/128,K/128), 输出Y(M,N)bf16]</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" t="n">
-        <v>58</v>
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>bf16 GEMM (Cijk/LoRA)</t>
+        </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>void at::native::(anonymous namespace)::multi_tensor_apply</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>LoRA ~44M(多小张量)</t>
-        </is>
-      </c>
-      <c r="D62" t="n">
-        <v>10</v>
-      </c>
-      <c r="E62" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="F62" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>memory</t>
-        </is>
-      </c>
-      <c r="H62" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I62" t="n">
-        <v>0</v>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>AdamW foreach(launch-bound)</t>
+          <t>shape=M×N×K;实参=[A(M,K), B(K,N)],输出(M,N);LoRA rank=16(N 或 K=16)</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" t="n">
-        <v>59</v>
+      <c r="A63" s="3" t="inlineStr">
+        <is>
+          <t>attention (attn_fwd/bwd)</t>
+        </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>void at::native::(anonymous namespace)::multi_tensor_apply</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>LoRA ~44M(多小张量)</t>
-        </is>
-      </c>
-      <c r="D63" t="n">
-        <v>11</v>
-      </c>
-      <c r="E63" t="n">
-        <v>0.11</v>
-      </c>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>memory</t>
-        </is>
-      </c>
-      <c r="H63" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I63" t="n">
-        <v>0</v>
-      </c>
-      <c r="J63" t="inlineStr">
-        <is>
-          <t>AdamW foreach(launch-bound)</t>
+          <t>q[1,32,2048,128] / k,v[1,8,2048,128](GQA 32/8,head_dim=128),causal,seq=2048</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>RCCL 通信</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>AG=参数 all-gather(bf16,每rank收 ≈14.4GB), RS=LoRA 梯度 reduce-scatter(≈0.6GB)</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>shape 含义图例</t>
+          <t>elementwise</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>对激活 [1,2048,4096] 或 FFN [1,2048,12288] 的逐元素(RMSNorm/残差/SwiGLU/scale/cast/copy);预估按第一个张量(4096)算,FFN 部分会偏低 → ≈</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>FP8 GEMM (ck::kernel_gemm)</t>
+          <t>量化 kernel</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>shape=M×N×K (M=2048,N/K∈{4096,12288,1024,151936});实参=[激活X(M,K)fp8, 权重W(N,K)fp8, 激活scale(M,K/128), 权重scale(N/128,K/128), 输出Y(M,N)bf16]</t>
+          <t>把激活/梯度 [2048,4096]或[2048,12288] 量化成 fp8+scale;1×128=按 token×128K, 128×1=按 128token×1</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>bf16 GEMM (Cijk/LoRA)</t>
+          <t>split_with_sizes_copy</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>shape=M×N×K;实参=[A(M,K), B(K,N)],输出(M,N);LoRA rank=16(N 或 K=16)</t>
+          <t>[8, 24269856]=8卡参数分片,all-gather 后解包成各 param view</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>attention (attn_fwd/bwd)</t>
+          <t>⚠访存预估口径</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>q[1,32,2048,128] / k,v[1,8,2048,128](GQA 32/8,head_dim=128),causal,seq=2048</t>
+          <t>访存型预估 = 按 shape 第一个张量 bytes/HBM,是【下限】;会低估 FFN(12288)与多操作数(mul/add)算子,故这些行的「实测/预估」偏大、不代表真实 headroom。可靠的 roofline 对比看 compute(GEMM/attn)与 comm。multi_tensor(AdamW) 为 launch-bound,不给 roofline。</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>RCCL 通信</t>
+          <t>数字含义</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
-        <is>
-          <t>AG=参数 all-gather(bf16,每rank收 ≈14.4GB), RS=LoRA 梯度 reduce-scatter(≈0.6GB)</t>
-        </is>
-      </c>
-    </row>
-    <row r="70">
-      <c r="A70" s="3" t="inlineStr">
-        <is>
-          <t>elementwise</t>
-        </is>
-      </c>
-      <c r="B70" t="inlineStr">
-        <is>
-          <t>对激活 [1,2048,4096] 或 FFN [1,2048,12288] 的逐元素(RMSNorm/残差/SwiGLU/scale/cast/copy);预估按第一个张量(4096)算,FFN 部分会偏低 → ≈</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" s="3" t="inlineStr">
-        <is>
-          <t>量化 kernel</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>把激活/梯度 [2048,4096]或[2048,12288] 量化成 fp8+scale;1×128=按 token×128K, 128×1=按 128token×1</t>
-        </is>
-      </c>
-    </row>
-    <row r="72">
-      <c r="A72" s="3" t="inlineStr">
-        <is>
-          <t>split_with_sizes_copy</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>[8, 24269856]=8卡参数分片,all-gather 后解包成各 param view</t>
-        </is>
-      </c>
-    </row>
-    <row r="73">
-      <c r="A73" s="3" t="inlineStr">
-        <is>
-          <t>⚠访存预估口径</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>访存型预估 = 按 shape 第一个张量 bytes/HBM,是【下限】;会低估 FFN(12288)与多操作数(mul/add)算子,故这些行的「实测/预估」偏大、不代表真实 headroom。可靠的 roofline 对比看 compute(GEMM/attn)与 comm。multi_tensor(AdamW) 为 launch-bound,不给 roofline。</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="3" t="inlineStr">
-        <is>
-          <t>数字含义</t>
-        </is>
-      </c>
-      <c r="B74" t="inlineStr">
         <is>
           <t>M=2048=本rank token数=MBS(1)×seq(2048);4096=hidden;12288=FFN中间维;1024=KV(GQA);128=head_dim/block;151936=vocab</t>
         </is>

</xml_diff>

<commit_message>
qwen3 perf docs: update to 568 ms best (GEMM tune + zero-copy RoPE)
</commit_message>
<xml_diff>
--- a/examples/qwen3/results/qwen3_fsdp2_operator_breakdown.xlsx
+++ b/examples/qwen3/results/qwen3_fsdp2_operator_breakdown.xlsx
@@ -453,7 +453,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>来源: chrome trace (step 15-17, 3 steps) | 8×MI308X | GPU kernel self-time. param-storage wall≈1419ms (GPU self 1548ms/step); best wall≈634ms (AITER attn+融合RMSNorm/RoPE) (GPU self 657ms/step)</t>
+          <t>来源: chrome trace (step 15-17, 3 steps) | 8×MI308X | GPU kernel self-time. param-storage wall≈1419ms (GPU self 1548ms/step); best wall≈603ms (AITER attn+融合RMSNorm/RoPE + RMSNorm-bwd large-M-small-N kernel) (GPU self 629ms/step)</t>
         </is>
       </c>
     </row>
@@ -637,10 +637,10 @@
         <v>435</v>
       </c>
       <c r="E11" t="n">
-        <v>42.2</v>
+        <v>14.1</v>
       </c>
       <c r="F11" t="n">
-        <v>42.2</v>
+        <v>14.1</v>
       </c>
     </row>
     <row r="12">
@@ -785,10 +785,10 @@
         <v>1547.7</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>657.4</v>
+        <v>629.3</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>-890.3</v>
+        <v>-918.4</v>
       </c>
     </row>
   </sheetData>
@@ -1514,7 +1514,7 @@
         <v>145</v>
       </c>
       <c r="F29" t="n">
-        <v>36.4</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="30">
@@ -1888,7 +1888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A9"/>
+  <dimension ref="A1:A10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -1953,7 +1953,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>结论: param-storage 是给 70B 防 OOM 的; 8B 最快 = cache+shard_grad_op+no-ckpt+bpreshuffle+AITER attn+融合RMSNorm/RoPE (634ms)。</t>
+          <t>结论: param-storage 是给 70B 防 OOM 的; 8B 最快(本表快照)= cache+shard_grad_op+no-ckpt+bpreshuffle+AITER attn+融合RMSNorm/RoPE (634ms)。叠加后续三项(见下)后达 568ms。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>后续优化(本 per-kernel 表为 634-config 的 trace 快照,以下进一步降到 568ms,详见 qwen3_fp8_perf_notes.md): ① RMSNorm 反向 large-M-small-N kernel 37.2-&gt;9.1ms (603ms); ② gfx942 bpreshuffle GEMM tune,FP8 GEMM 295-&gt;277ms (578ms); ③ zero-copy RoPE 布局,去掉~2.3GB/step contiguous 拷贝 (568ms)。</t>
         </is>
       </c>
     </row>
@@ -2831,7 +2838,7 @@
         <v>145</v>
       </c>
       <c r="E10" t="n">
-        <v>36.35</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="F10" t="n">
         <v>0.92</v>
@@ -2843,15 +2850,15 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>39.60x</t>
+          <t>9.0x</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>5.6</v>
+        <v>1.4</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>融合 RMSNorm 反向(dX+dW)</t>
+          <t>融合 RMSNorm 反向(dX+dW); large-M-small-N 行并行特化</t>
         </is>
       </c>
     </row>

</xml_diff>